<commit_message>
AI handle return request triage into real workflow + skip SB enqueue on rejects + move agent shutdown to agent.py
</commit_message>
<xml_diff>
--- a/return_orders.xlsx
+++ b/return_orders.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preci\ReturnAppProj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777CCB7D-2D4A-45DE-ADC2-90F228590250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E32F2A-7A81-41A5-95FC-8477814CD29C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,10 +89,10 @@
     <t>Pending</t>
   </si>
   <si>
+    <t>221B Baker St, London W1U 6QQ</t>
+  </si>
+  <si>
     <t>damaged</t>
-  </si>
-  <si>
-    <t>221B Baker St, London W1U 6QQ</t>
   </si>
 </sst>
 </file>
@@ -535,13 +535,13 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
       </c>
       <c r="G2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H2" t="s">
         <v>16</v>

</xml_diff>